<commit_message>
Thêm cột so sánh với kỳ trả cổ tức tiền mặt gần nhất
- _cash_history + _compare_prev: lấy kỳ cổ tức tiền mặt gần nhất trước đó
- 3 cột mới: Cổ tức TM kỳ trước, Ngày kỳ trước, So với kỳ trước (Tăng/Giảm/Bằng)
- dữ liệu từ chính nguồn vnstock (không cần Vietstock)
</commit_message>
<xml_diff>
--- a/data/lich_su_kien.xlsx
+++ b/data/lich_su_kien.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,11 +484,26 @@
           <t>Ngày thực hiện</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Cổ tức TM kỳ trước (đ/cp)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Ngày kỳ trước</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>So với kỳ trước</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MWG</t>
+          <t>REE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -498,7 +513,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CTCP Đầu tư Thế giới Di động</t>
+          <t>CTCP Cơ Điện Lạnh</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -513,31 +528,34 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MWG - Tổ chức ĐHĐCĐ thường niên 2026</t>
+          <t>REE - Tổ chức ĐHĐCĐ thường niên 2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
-        </is>
-      </c>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HPG</t>
+          <t>REE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -547,46 +565,67 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CTCP Tập đoàn Hòa Phát</t>
+          <t>CTCP Cơ Điện Lạnh</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ĐHĐCĐ / Lấy ý kiến</t>
+          <t>Cổ tức / Phát hành</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Đại hội Đồng Cổ đông</t>
+          <t>Trả cổ tức bằng tiền mặt</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>HPG - Tổ chức ĐHĐCĐ thường niên 2026</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+          <t>Trả cổ tức bằng tiền mặt - Đợt 1 2025 - 1,000 VND</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1000</v>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2025-02-27</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Bằng (1000)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PNJ</t>
+          <t>FPT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -596,7 +635,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CTCP Vàng bạc Đá quý Phú Nhuận</t>
+          <t>CTCP FPT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -611,26 +650,29 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PNJ - Tổ chức ĐHĐCĐ thường niên 2026</t>
+          <t>FPT - Tổ chức ĐHĐCĐ thường niên 2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -680,11 +722,14 @@
           <t>2026-04-22</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DGC</t>
+          <t>REE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -694,46 +739,49 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CTCP Tập đoàn Hóa chất Đức Giang</t>
+          <t>CTCP Cơ Điện Lạnh</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ĐHĐCĐ / Lấy ý kiến</t>
+          <t>Cổ tức / Phát hành</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Đại hội Cổ đông Bất thường</t>
+          <t>Phát hành cổ phiếu</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DGC - Tổ chức ĐHĐCĐ bất thường 2026</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Phát hành cổ phiếu - Trả Cổ tức bằng Cổ phiếu tỉ lệ 15.0%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PNJ</t>
+          <t>FPT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -743,7 +791,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CTCP Vàng bạc Đá quý Phú Nhuận</t>
+          <t>CTCP FPT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -753,36 +801,57 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Phát hành cổ phiếu</t>
+          <t>Trả cổ tức bằng tiền mặt</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Phát hành cổ phiếu - Cổ phiếu thưởng tỉ lệ 50.0%</t>
+          <t>Trả cổ tức bằng tiền mặt - Đợt 2 2025 - 1,000 VND</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1000</v>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Bằng (1000)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HPG</t>
+          <t>FPT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -792,7 +861,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CTCP Tập đoàn Hòa Phát</t>
+          <t>CTCP FPT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -802,42 +871,31 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Trả cổ tức bằng tiền mặt</t>
+          <t>Phát hành cổ phiếu</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Trả cổ tức bằng tiền mặt - Cả năm 2025 - 500 VND</t>
+          <t>Phát hành cổ phiếu - Phát hành cho CBCNV tỉ lệ 0.5%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>500</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
+          <t>0.499%</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HPG</t>
+          <t>FPT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -847,7 +905,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CTCP Tập đoàn Hòa Phát</t>
+          <t>CTCP FPT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -862,7 +920,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Phát hành cổ phiếu - Trả Cổ tức bằng Cổ phiếu tỉ lệ 10.0%</t>
+          <t>Phát hành cổ phiếu - Cổ phiếu thưởng tỉ lệ 10.0%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -871,22 +929,17 @@
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FPT</t>
+          <t>REE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -896,7 +949,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CTCP FPT</t>
+          <t>CTCP Cơ Điện Lạnh</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -906,242 +959,26 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Trả cổ tức bằng tiền mặt</t>
+          <t>Phát hành cổ phiếu</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Trả cổ tức bằng tiền mặt - Đợt 2 2025 - 1,000 VND</t>
+          <t>Phát hành cổ phiếu - Phát hành cho CBCNV tỉ lệ 0.1%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>FPT</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>HOSE</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CTCP FPT</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Cổ tức / Phát hành</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu - Phát hành cho CBCNV tỉ lệ 0.5%</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>0.499%</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>FPT</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>HOSE</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>CTCP FPT</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Cổ tức / Phát hành</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu - Cổ phiếu thưởng tỉ lệ 10.0%</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>MWG</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>HOSE</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>CTCP Đầu tư Thế giới Di động</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Cổ tức / Phát hành</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu - Phát hành cho CBCNV tỉ lệ 0.2%</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>0.2%</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>MWG</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>HOSE</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>CTCP Đầu tư Thế giới Di động</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Cổ tức / Phát hành</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu - Phát hành cho CBCNV tỉ lệ 0.5%</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>0.5%</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PNJ</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>HOSE</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>CTCP Vàng bạc Đá quý Phú Nhuận</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Cổ tức / Phát hành</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Phát hành cổ phiếu - Phát hành cho CBCNV tỉ lệ 0.7%</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>0.7%</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+          <t>0.09%</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>